<commit_message>
feat: Implement license management system, vacation reports, and company creation wizard with core application and database updates.
</commit_message>
<xml_diff>
--- a/public/template_empleados.xlsx
+++ b/public/template_empleados.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="176">
   <si>
     <t>CÓDIGO EMPLEADO*</t>
   </si>
@@ -265,112 +265,100 @@
     <t>CARGO</t>
   </si>
   <si>
-    <t>ADMINISTRATIVE ASSISTANT</t>
+    <t>GERENCIA</t>
+  </si>
+  <si>
+    <t>OPERATIVO</t>
+  </si>
+  <si>
+    <t>FUNCIÓN</t>
   </si>
   <si>
     <t>CEO</t>
   </si>
   <si>
-    <t>HELP DESK MANAGER</t>
-  </si>
-  <si>
-    <t>HELP DESK SUPPORT</t>
-  </si>
-  <si>
-    <t>PROGRAMADOR SENIOR</t>
-  </si>
-  <si>
-    <t>SALES MANAGER</t>
-  </si>
-  <si>
-    <t>FUNCIÓN</t>
-  </si>
-  <si>
-    <t>ASISTENTE ADMINISTRATIVO</t>
-  </si>
-  <si>
-    <t>GERENTE DE VENTAS</t>
-  </si>
-  <si>
-    <t>SOPORTE TECNICO</t>
+    <t>GERENTE</t>
+  </si>
+  <si>
+    <t>TECNICO</t>
   </si>
   <si>
     <t>PARTIDA</t>
   </si>
   <si>
-    <t xml:space="preserve">2.10.12.001. - </t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.10.12.002. - </t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.10.12.005. - </t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.10.12.010. - </t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.10.12.011. - </t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.10.12.012. - </t>
-  </si>
-  <si>
-    <t xml:space="preserve">6.10.10.001. - </t>
-  </si>
-  <si>
-    <t xml:space="preserve">6.10.10.002. - </t>
-  </si>
-  <si>
-    <t xml:space="preserve">6.10.10.003. - </t>
-  </si>
-  <si>
-    <t xml:space="preserve">6.10.10.004. - </t>
-  </si>
-  <si>
-    <t xml:space="preserve">6.10.10.007. - </t>
-  </si>
-  <si>
-    <t xml:space="preserve">6.10.10.008. - </t>
-  </si>
-  <si>
-    <t xml:space="preserve">6.10.10.009. - </t>
-  </si>
-  <si>
-    <t xml:space="preserve">6.10.10.010. - </t>
-  </si>
-  <si>
-    <t xml:space="preserve">6.10.10.012. - </t>
-  </si>
-  <si>
-    <t xml:space="preserve">6.10.10.013. - </t>
-  </si>
-  <si>
-    <t xml:space="preserve">6.10.10.019. - </t>
-  </si>
-  <si>
-    <t xml:space="preserve">6.10.10.020. - </t>
-  </si>
-  <si>
-    <t xml:space="preserve">6.10.10.021. - </t>
-  </si>
-  <si>
-    <t xml:space="preserve">6.10.10.024. - </t>
-  </si>
-  <si>
-    <t xml:space="preserve">6.10.15.002. - </t>
-  </si>
-  <si>
-    <t xml:space="preserve">6.10.15.004. - </t>
-  </si>
-  <si>
-    <t xml:space="preserve">6.10.15.011. - </t>
-  </si>
-  <si>
-    <t xml:space="preserve">6.10.15.012. - </t>
-  </si>
-  <si>
-    <t xml:space="preserve">6.10.99. - </t>
+    <t>2.10.12.001. - Seguro social por pagar</t>
+  </si>
+  <si>
+    <t>2.10.12.002. - Salarios por pagar</t>
+  </si>
+  <si>
+    <t>2.10.12.005. - Imp. sobre la renta por pagar</t>
+  </si>
+  <si>
+    <t>2.10.12.010. - Seguro educativo por pagar</t>
+  </si>
+  <si>
+    <t>2.10.12.011. - Seguro riesgo profesional por pagar</t>
+  </si>
+  <si>
+    <t>2.10.12.012. - Decimo tercer mes por pagar</t>
+  </si>
+  <si>
+    <t>6.10.10.001. - Sueldos</t>
+  </si>
+  <si>
+    <t>6.10.10.002. - Horas extras</t>
+  </si>
+  <si>
+    <t>6.10.10.003. - Vacaciones</t>
+  </si>
+  <si>
+    <t>6.10.10.004. - Xii mes</t>
+  </si>
+  <si>
+    <t>6.10.10.007. - Gasto de representacion</t>
+  </si>
+  <si>
+    <t>6.10.10.008. - Xiii gasto de representacion</t>
+  </si>
+  <si>
+    <t>6.10.10.009. - Viatico</t>
+  </si>
+  <si>
+    <t>6.10.10.010. - Bonificacion</t>
+  </si>
+  <si>
+    <t>6.10.10.012. - Prima de antiguedad</t>
+  </si>
+  <si>
+    <t>6.10.10.013. - Indemnizacion</t>
+  </si>
+  <si>
+    <t>6.10.10.019. - Seguro social patronal</t>
+  </si>
+  <si>
+    <t>6.10.10.020. - Seguro educativo patronal</t>
+  </si>
+  <si>
+    <t>6.10.10.021. - Seguro riesgo profesional</t>
+  </si>
+  <si>
+    <t>6.10.10.024. - Recargos seguro social</t>
+  </si>
+  <si>
+    <t>6.10.15.002. - Honorarios de contabilidad</t>
+  </si>
+  <si>
+    <t>6.10.15.004. - Honorarios por soporte tecnico</t>
+  </si>
+  <si>
+    <t>6.10.15.011. - Honorarios por desarrollo</t>
+  </si>
+  <si>
+    <t>6.10.15.012. - Honorarios por administracion</t>
+  </si>
+  <si>
+    <t>6.10.99. - IMPUESTO SOBRE LA RENTA</t>
   </si>
   <si>
     <t>ORGANIGRAMA</t>
@@ -379,16 +367,7 @@
     <t>ADMINISTRACIÓN</t>
   </si>
   <si>
-    <t>DESARROLLO</t>
-  </si>
-  <si>
     <t>DIRECCIÓN GENERAL</t>
-  </si>
-  <si>
-    <t>SOPORTE TÉCNICO</t>
-  </si>
-  <si>
-    <t>VENTAS</t>
   </si>
   <si>
     <t>INSTRUCCIONES PARA IMPORTAR EMPLEADOS</t>
@@ -1284,7 +1263,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:C53"/>
+  <dimension ref="A1:C44"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="true" style="0"/>
@@ -1429,7 +1408,7 @@
         <v>81</v>
       </c>
       <c r="B13">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C13" t="s">
         <v>82</v>
@@ -1440,7 +1419,7 @@
         <v>81</v>
       </c>
       <c r="B14">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="C14" t="s">
         <v>83</v>
@@ -1448,46 +1427,46 @@
     </row>
     <row r="15" spans="1:3">
       <c r="A15" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B15">
         <v>3</v>
       </c>
       <c r="C15" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="16" spans="1:3">
       <c r="A16" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B16">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C16" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B17">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="C17" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="B18">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="C18" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="19" spans="1:3">
@@ -1495,10 +1474,10 @@
         <v>88</v>
       </c>
       <c r="B19">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="C19" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="20" spans="1:3">
@@ -1506,10 +1485,10 @@
         <v>88</v>
       </c>
       <c r="B20">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="C20" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
     </row>
     <row r="21" spans="1:3">
@@ -1517,10 +1496,10 @@
         <v>88</v>
       </c>
       <c r="B21">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="C21" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="22" spans="1:3">
@@ -1528,10 +1507,10 @@
         <v>88</v>
       </c>
       <c r="B22">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="C22" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
     </row>
     <row r="23" spans="1:3">
@@ -1539,340 +1518,241 @@
         <v>88</v>
       </c>
       <c r="B23">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="C23" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="B24">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="C24" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="B25">
-        <v>16</v>
+        <v>3</v>
       </c>
       <c r="C25" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="B26">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="C26" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="B27">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="C27" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="28" spans="1:3">
       <c r="A28" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="B28">
-        <v>19</v>
+        <v>5</v>
       </c>
       <c r="C28" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="29" spans="1:3">
       <c r="A29" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="B29">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="C29" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="30" spans="1:3">
       <c r="A30" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="B30">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="C30" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="31" spans="1:3">
       <c r="A31" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="B31">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C31" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="32" spans="1:3">
       <c r="A32" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="B32">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="C32" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
     </row>
     <row r="33" spans="1:3">
       <c r="A33" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="B33">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="C33" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
     </row>
     <row r="34" spans="1:3">
       <c r="A34" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="B34">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="C34" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
     </row>
     <row r="35" spans="1:3">
       <c r="A35" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="B35">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="C35" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
     </row>
     <row r="36" spans="1:3">
       <c r="A36" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="B36">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="C36" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
     </row>
     <row r="37" spans="1:3">
       <c r="A37" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="B37">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="C37" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="38" spans="1:3">
       <c r="A38" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="B38">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="C38" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
     <row r="39" spans="1:3">
       <c r="A39" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="B39">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="C39" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="40" spans="1:3">
       <c r="A40" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="B40">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="C40" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
     </row>
     <row r="41" spans="1:3">
       <c r="A41" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="B41">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="C41" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="42" spans="1:3">
       <c r="A42" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="B42">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="C42" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="43" spans="1:3">
       <c r="A43" t="s">
-        <v>92</v>
+        <v>114</v>
       </c>
       <c r="B43">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="C43" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
     </row>
     <row r="44" spans="1:3">
       <c r="A44" t="s">
-        <v>92</v>
+        <v>114</v>
       </c>
       <c r="B44">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="C44" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3">
-      <c r="A45" t="s">
-        <v>92</v>
-      </c>
-      <c r="B45">
-        <v>23</v>
-      </c>
-      <c r="C45" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3">
-      <c r="A46" t="s">
-        <v>92</v>
-      </c>
-      <c r="B46">
-        <v>24</v>
-      </c>
-      <c r="C46" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3">
-      <c r="A47" t="s">
-        <v>92</v>
-      </c>
-      <c r="B47">
-        <v>25</v>
-      </c>
-      <c r="C47" t="s">
         <v>116</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3">
-      <c r="A48" t="s">
-        <v>92</v>
-      </c>
-      <c r="B48">
-        <v>21</v>
-      </c>
-      <c r="C48" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3">
-      <c r="A49" t="s">
-        <v>118</v>
-      </c>
-      <c r="B49">
-        <v>8</v>
-      </c>
-      <c r="C49" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3">
-      <c r="A50" t="s">
-        <v>118</v>
-      </c>
-      <c r="B50">
-        <v>7</v>
-      </c>
-      <c r="C50" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3">
-      <c r="A51" t="s">
-        <v>118</v>
-      </c>
-      <c r="B51">
-        <v>1</v>
-      </c>
-      <c r="C51" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3">
-      <c r="A52" t="s">
-        <v>118</v>
-      </c>
-      <c r="B52">
-        <v>2</v>
-      </c>
-      <c r="C52" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3">
-      <c r="A53" t="s">
-        <v>118</v>
-      </c>
-      <c r="B53">
-        <v>6</v>
-      </c>
-      <c r="C53" t="s">
-        <v>123</v>
       </c>
     </row>
   </sheetData>
@@ -1904,7 +1784,7 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
     </row>
     <row r="2" spans="1:1">
@@ -1912,57 +1792,57 @@
     </row>
     <row r="3" spans="1:1">
       <c r="A3" t="s">
-        <v>125</v>
+        <v>118</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" t="s">
-        <v>128</v>
+        <v>121</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
     </row>
     <row r="9" spans="1:1">
       <c r="A9" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
     </row>
     <row r="10" spans="1:1">
       <c r="A10" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
     </row>
     <row r="11" spans="1:1">
       <c r="A11" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
     </row>
     <row r="12" spans="1:1">
       <c r="A12" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
     </row>
     <row r="13" spans="1:1">
       <c r="A13" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
     </row>
     <row r="14" spans="1:1">
@@ -1970,42 +1850,42 @@
     </row>
     <row r="15" spans="1:1">
       <c r="A15" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
     </row>
     <row r="16" spans="1:1">
       <c r="A16" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
     </row>
     <row r="17" spans="1:1">
       <c r="A17" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
     </row>
     <row r="18" spans="1:1">
       <c r="A18" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
     </row>
     <row r="19" spans="1:1">
       <c r="A19" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
     </row>
     <row r="20" spans="1:1">
       <c r="A20" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
     </row>
     <row r="21" spans="1:1">
       <c r="A21" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
     </row>
     <row r="22" spans="1:1">
       <c r="A22" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
     </row>
     <row r="23" spans="1:1">
@@ -2013,17 +1893,17 @@
     </row>
     <row r="24" spans="1:1">
       <c r="A24" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
     </row>
     <row r="25" spans="1:1">
       <c r="A25" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
     </row>
     <row r="26" spans="1:1">
       <c r="A26" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
     </row>
     <row r="27" spans="1:1">
@@ -2031,37 +1911,37 @@
     </row>
     <row r="28" spans="1:1">
       <c r="A28" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
     </row>
     <row r="29" spans="1:1">
       <c r="A29" t="s">
-        <v>148</v>
+        <v>141</v>
       </c>
     </row>
     <row r="30" spans="1:1">
       <c r="A30" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
     </row>
     <row r="31" spans="1:1">
       <c r="A31" t="s">
-        <v>150</v>
+        <v>143</v>
       </c>
     </row>
     <row r="32" spans="1:1">
       <c r="A32" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
     </row>
     <row r="33" spans="1:1">
       <c r="A33" t="s">
-        <v>152</v>
+        <v>145</v>
       </c>
     </row>
     <row r="34" spans="1:1">
       <c r="A34" t="s">
-        <v>153</v>
+        <v>146</v>
       </c>
     </row>
     <row r="35" spans="1:1">
@@ -2069,7 +1949,7 @@
     </row>
     <row r="36" spans="1:1">
       <c r="A36" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
     </row>
     <row r="37" spans="1:1">
@@ -2077,42 +1957,42 @@
     </row>
     <row r="38" spans="1:1">
       <c r="A38" t="s">
-        <v>155</v>
+        <v>148</v>
       </c>
     </row>
     <row r="39" spans="1:1">
       <c r="A39" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
     </row>
     <row r="40" spans="1:1">
       <c r="A40" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
     </row>
     <row r="41" spans="1:1">
       <c r="A41" t="s">
-        <v>158</v>
+        <v>151</v>
       </c>
     </row>
     <row r="42" spans="1:1">
       <c r="A42" t="s">
-        <v>159</v>
+        <v>152</v>
       </c>
     </row>
     <row r="43" spans="1:1">
       <c r="A43" t="s">
-        <v>160</v>
+        <v>153</v>
       </c>
     </row>
     <row r="44" spans="1:1">
       <c r="A44" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
     </row>
     <row r="45" spans="1:1">
       <c r="A45" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
     </row>
     <row r="46" spans="1:1">
@@ -2120,27 +2000,27 @@
     </row>
     <row r="47" spans="1:1">
       <c r="A47" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
     </row>
     <row r="48" spans="1:1">
       <c r="A48" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
     </row>
     <row r="49" spans="1:1">
       <c r="A49" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
     </row>
     <row r="50" spans="1:1">
       <c r="A50" t="s">
-        <v>166</v>
+        <v>159</v>
       </c>
     </row>
     <row r="51" spans="1:1">
       <c r="A51" t="s">
-        <v>167</v>
+        <v>160</v>
       </c>
     </row>
     <row r="52" spans="1:1">
@@ -2148,42 +2028,42 @@
     </row>
     <row r="53" spans="1:1">
       <c r="A53" t="s">
-        <v>168</v>
+        <v>161</v>
       </c>
     </row>
     <row r="54" spans="1:1">
       <c r="A54" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
     </row>
     <row r="55" spans="1:1">
       <c r="A55" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
     </row>
     <row r="56" spans="1:1">
       <c r="A56" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
     </row>
     <row r="57" spans="1:1">
       <c r="A57" t="s">
-        <v>172</v>
+        <v>165</v>
       </c>
     </row>
     <row r="58" spans="1:1">
       <c r="A58" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
     </row>
     <row r="59" spans="1:1">
       <c r="A59" t="s">
-        <v>174</v>
+        <v>167</v>
       </c>
     </row>
     <row r="60" spans="1:1">
       <c r="A60" t="s">
-        <v>175</v>
+        <v>168</v>
       </c>
     </row>
     <row r="61" spans="1:1">
@@ -2191,37 +2071,37 @@
     </row>
     <row r="62" spans="1:1">
       <c r="A62" t="s">
-        <v>176</v>
+        <v>169</v>
       </c>
     </row>
     <row r="63" spans="1:1">
       <c r="A63" t="s">
-        <v>177</v>
+        <v>170</v>
       </c>
     </row>
     <row r="64" spans="1:1">
       <c r="A64" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
     </row>
     <row r="65" spans="1:1">
       <c r="A65" t="s">
-        <v>179</v>
+        <v>172</v>
       </c>
     </row>
     <row r="66" spans="1:1">
       <c r="A66" t="s">
-        <v>180</v>
+        <v>173</v>
       </c>
     </row>
     <row r="67" spans="1:1">
       <c r="A67" t="s">
-        <v>181</v>
+        <v>174</v>
       </c>
     </row>
     <row r="68" spans="1:1">
       <c r="A68" t="s">
-        <v>182</v>
+        <v>175</v>
       </c>
     </row>
   </sheetData>

</xml_diff>